<commit_message>
created save informarion state on excel
</commit_message>
<xml_diff>
--- a/CedulasRut.xlsx
+++ b/CedulasRut.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juang\OneDrive\Documentos\ARCHIVOSDIAN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\RPAv1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A06CC2-B614-487E-97A2-56C3426E3C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60449AC6-E2E2-46B8-A43E-7C51D50891EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cedulas" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" fullCalcOnLoad="1" fullPrecision="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,16 +25,29 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>identificacion</t>
   </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>No está inscrito en el RUT</t>
+  </si>
+  <si>
+    <t>registro activo</t>
+  </si>
+  <si>
+    <t>resultado desconocido</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -345,28 +358,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2">
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
         <v>1146442202</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="B2" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
         <v>1035234348</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>15527721</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>1020457875</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>1000203619</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>94521440</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>1017134896</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>71630403</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>14973980</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>43285731</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>1</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>2</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>3</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>98042654248</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
+</file>
+
+<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to RpaBot under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
+For more information about EPPlus, see https://epplussoftware.com/
+
 </file>
</xml_diff>

<commit_message>
prueba con 30 registros
</commit_message>
<xml_diff>
--- a/CedulasRut.xlsx
+++ b/CedulasRut.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\RPAv1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60449AC6-E2E2-46B8-A43E-7C51D50891EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EB50B7-11B8-4DA1-85C1-55175E4DEE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>identificacion</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>resultado desconocido</t>
+  </si>
+  <si>
+    <t>registro cancelado</t>
   </si>
 </sst>
 </file>
@@ -358,7 +361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="12" customWidth="1"/>
@@ -417,7 +420,7 @@
         <v>94521440</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -482,6 +485,521 @@
       </c>
       <c r="B15" s="0" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>4</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>5</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>6</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>7</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>8</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>9</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>10</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>11</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>12</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>13</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>14</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>15</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>16</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>17</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>18</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>19</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>20</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>21</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0">
+        <v>22</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>23</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>24</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0">
+        <v>25</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0">
+        <v>26</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0">
+        <v>27</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0">
+        <v>28</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0">
+        <v>29</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
+        <v>30</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0">
+        <v>31</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0">
+        <v>32</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0">
+        <v>33</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>